<commit_message>
Aula 5 finaliza, modificação Readme com check de aulas, modificação arquivos anteriores, para remoção de subtitulo de sumário
</commit_message>
<xml_diff>
--- a/Analise_de_dados_e_IA_Nivelamento/Semana_01/Excel/03_Formulas_e_Funcoes/src/Meteora Ecommerce - FINAL AULA 2.xlsx
+++ b/Analise_de_dados_e_IA_Nivelamento/Semana_01/Excel/03_Formulas_e_Funcoes/src/Meteora Ecommerce - FINAL AULA 2.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Thierry-G15\Documents\Estudos\Alura\Santander-Imersao-Digital\Analise_de_dados_e_IA_Nivelamento\Semana_01\Excel\03_Formulas_e_Funcoes\src\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{6F53CABF-D26D-4840-B230-B5FF05DC2B3E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5DD64933-9B0A-4466-A984-7479D48D933F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-28920" yWindow="-4080" windowWidth="29040" windowHeight="15720" xr2:uid="{F6D97A53-F63B-4272-A181-44B26E0B790F}"/>
+    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" activeTab="1" xr2:uid="{F6D97A53-F63B-4272-A181-44B26E0B790F}"/>
   </bookViews>
   <sheets>
     <sheet name="Produtos" sheetId="1" r:id="rId1"/>
@@ -35,7 +35,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="127" uniqueCount="24">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="135" uniqueCount="31">
   <si>
     <t>Produtos</t>
   </si>
@@ -107,6 +107,27 @@
   </si>
   <si>
     <t>Total</t>
+  </si>
+  <si>
+    <t>Valor total</t>
+  </si>
+  <si>
+    <t>Totais</t>
+  </si>
+  <si>
+    <t>Desconto</t>
+  </si>
+  <si>
+    <t>Valor Desconto</t>
+  </si>
+  <si>
+    <t>Valor Total</t>
+  </si>
+  <si>
+    <t>Valor  desconto</t>
+  </si>
+  <si>
+    <t>5%</t>
   </si>
 </sst>
 </file>
@@ -117,7 +138,7 @@
     <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
     <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
   </numFmts>
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -144,6 +165,13 @@
       <b/>
       <sz val="14"/>
       <color theme="0" tint="-4.9989318521683403E-2"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <sz val="11"/>
+      <color theme="1"/>
       <name val="Calibri"/>
       <family val="2"/>
       <scheme val="minor"/>
@@ -175,7 +203,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="20">
     <border>
       <left/>
       <right/>
@@ -214,16 +242,31 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
+      <left style="medium">
         <color indexed="64"/>
       </left>
-      <right style="medium">
+      <right style="thin">
         <color indexed="64"/>
       </right>
       <top style="thin">
         <color indexed="64"/>
       </top>
-      <bottom style="thin">
+      <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -235,7 +278,7 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
@@ -250,10 +293,25 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
       <bottom style="medium">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -262,13 +320,28 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom style="thin">
+        <color indexed="64"/>
+      </bottom>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
       <right style="medium">
         <color indexed="64"/>
       </right>
-      <top style="thin">
+      <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
+      <bottom style="thin">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -280,8 +353,69 @@
       <right style="thin">
         <color indexed="64"/>
       </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="medium">
+        <color indexed="64"/>
+      </right>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="medium">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="thin">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
+      <top style="thin">
+        <color indexed="64"/>
+      </top>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left style="medium">
+        <color indexed="64"/>
+      </left>
+      <right style="thin">
+        <color indexed="64"/>
+      </right>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -294,7 +428,7 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
+      <bottom style="medium">
         <color indexed="64"/>
       </bottom>
       <diagonal/>
@@ -307,21 +441,6 @@
         <color indexed="64"/>
       </right>
       <top/>
-      <bottom style="thin">
-        <color indexed="64"/>
-      </bottom>
-      <diagonal/>
-    </border>
-    <border>
-      <left style="medium">
-        <color indexed="64"/>
-      </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
-      <top style="medium">
-        <color indexed="64"/>
-      </top>
       <bottom style="medium">
         <color indexed="64"/>
       </bottom>
@@ -331,37 +450,30 @@
       <left style="thin">
         <color indexed="64"/>
       </left>
-      <right style="thin">
-        <color indexed="64"/>
-      </right>
+      <right/>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
     <border>
-      <left style="thin">
-        <color indexed="64"/>
-      </left>
+      <left/>
       <right style="medium">
         <color indexed="64"/>
       </right>
       <top style="medium">
         <color indexed="64"/>
       </top>
-      <bottom style="medium">
-        <color indexed="64"/>
-      </bottom>
+      <bottom/>
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="1">
+  <cellStyleXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
+    <xf numFmtId="9" fontId="4" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="44">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center"/>
@@ -377,67 +489,355 @@
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="2" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="4" xfId="0" applyBorder="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="5" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="7" xfId="0" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="8" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="10" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="11" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
+    <xf numFmtId="165" fontId="3" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center"/>
+    </xf>
     <xf numFmtId="0" fontId="3" fillId="4" borderId="12" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="9" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="3" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="14" xfId="0" applyBorder="1"/>
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="6" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="15" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="16" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="right"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="16" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="16" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="6" xfId="0" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="17" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="18" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="13" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="19" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="165" fontId="0" fillId="3" borderId="9" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="4" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="8" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyBorder="1"/>
-    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
-    <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center"/>
-    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="9" fontId="0" fillId="3" borderId="0" xfId="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="left"/>
+    </xf>
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="14" xfId="0" applyNumberFormat="1" applyBorder="1"/>
+    <xf numFmtId="164" fontId="0" fillId="3" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
   </cellXfs>
-  <cellStyles count="1">
+  <cellStyles count="2">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
+    <cellStyle name="Porcentagem" xfId="1" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="15">
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
     </dxf>
     <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="14"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDAFF01"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
       <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDAFF01"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDAFF01"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <font>
+        <b val="0"/>
+        <i val="0"/>
+        <strike val="0"/>
+        <condense val="0"/>
+        <extend val="0"/>
+        <outline val="0"/>
+        <shadow val="0"/>
+        <u val="none"/>
+        <vertAlign val="baseline"/>
+        <sz val="11"/>
+        <color theme="1"/>
+        <name val="Calibri"/>
+        <family val="2"/>
+        <scheme val="minor"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor indexed="64"/>
+          <bgColor rgb="FFDAFF01"/>
+        </patternFill>
+      </fill>
+      <alignment horizontal="left" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="165" formatCode="&quot;R$&quot;\ #,##0.00"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical/>
+        <horizontal/>
+      </border>
+    </dxf>
+    <dxf>
+      <numFmt numFmtId="164" formatCode="_-[$R$-416]\ * #,##0.00_-;\-[$R$-416]\ * #,##0.00_-;_-[$R$-416]\ * &quot;-&quot;??_-;_-@_-"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="0" indent="0" justifyLastLine="0" shrinkToFit="0" readingOrder="0"/>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
+    </dxf>
+    <dxf>
+      <border diagonalUp="0" diagonalDown="0">
+        <left style="thin">
+          <color indexed="64"/>
+        </left>
+        <right style="thin">
+          <color indexed="64"/>
+        </right>
+        <top style="thin">
+          <color indexed="64"/>
+        </top>
+        <bottom style="thin">
+          <color indexed="64"/>
+        </bottom>
+        <vertical style="thin">
+          <color indexed="64"/>
+        </vertical>
+        <horizontal style="thin">
+          <color indexed="64"/>
+        </horizontal>
+      </border>
     </dxf>
     <dxf>
       <font>
@@ -477,16 +877,20 @@
 </file>
 
 <file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9DDBCA65-023C-4EC1-98AB-9D3EFD52E7AF}" name="Tabela5" displayName="Tabela5" ref="A3:E24" totalsRowCount="1" headerRowDxfId="5">
-  <autoFilter ref="A3:E23" xr:uid="{9DDBCA65-023C-4EC1-98AB-9D3EFD52E7AF}"/>
-  <tableColumns count="5">
-    <tableColumn id="1" xr3:uid="{0DC906EA-AFD4-4719-8B69-33FF19C2D8D0}" name="Produtos" totalsRowLabel="Total"/>
-    <tableColumn id="2" xr3:uid="{5868626F-6538-4792-A504-C58671A675E4}" name="Tamanho" dataDxfId="4" totalsRowDxfId="3"/>
-    <tableColumn id="3" xr3:uid="{D4BC101A-97D8-4654-894F-A95A0763ECFC}" name="Categoria"/>
-    <tableColumn id="4" xr3:uid="{34BA93BF-7C06-4A74-819A-029EE57FACDA}" name="Preço Unitário" totalsRowFunction="sum" dataDxfId="2"/>
-    <tableColumn id="5" xr3:uid="{79E8B5D8-9831-45EA-85F5-D3CD7A1F217D}" name="Qtd" totalsRowFunction="sum" dataDxfId="1" totalsRowDxfId="0"/>
+<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="5" xr:uid="{9DDBCA65-023C-4EC1-98AB-9D3EFD52E7AF}" name="Tabela5" displayName="Tabela5" ref="A3:G25" totalsRowCount="1" headerRowDxfId="14">
+  <autoFilter ref="A3:G24" xr:uid="{9DDBCA65-023C-4EC1-98AB-9D3EFD52E7AF}"/>
+  <tableColumns count="7">
+    <tableColumn id="1" xr3:uid="{0DC906EA-AFD4-4719-8B69-33FF19C2D8D0}" name="Produtos" totalsRowLabel="Desconto" dataDxfId="13" totalsRowDxfId="2"/>
+    <tableColumn id="2" xr3:uid="{5868626F-6538-4792-A504-C58671A675E4}" name="Tamanho" dataDxfId="12" totalsRowDxfId="1"/>
+    <tableColumn id="3" xr3:uid="{D4BC101A-97D8-4654-894F-A95A0763ECFC}" name="Categoria" dataDxfId="11" totalsRowDxfId="0"/>
+    <tableColumn id="4" xr3:uid="{34BA93BF-7C06-4A74-819A-029EE57FACDA}" name="Preço Unitário" totalsRowLabel="5%" dataDxfId="8" totalsRowDxfId="6" totalsRowCellStyle="Porcentagem"/>
+    <tableColumn id="5" xr3:uid="{79E8B5D8-9831-45EA-85F5-D3CD7A1F217D}" name="Qtd" dataDxfId="10" totalsRowDxfId="5"/>
+    <tableColumn id="6" xr3:uid="{0EF4DB0D-92F6-41E8-8FD8-078AF6BEC52F}" name="Valor Total" dataDxfId="9" totalsRowDxfId="4"/>
+    <tableColumn id="7" xr3:uid="{DB4F4E2C-739F-4F8C-A2E1-A1F3E2B9801F}" name="Valor  desconto" dataDxfId="7" totalsRowDxfId="3">
+      <calculatedColumnFormula>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</calculatedColumnFormula>
+    </tableColumn>
   </tableColumns>
-  <tableStyleInfo name="TableStyleLight8" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
+  <tableStyleInfo name="TableStyleMedium1" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </table>
 </file>
 
@@ -787,7 +1191,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{7162DC3F-8DD7-4F1A-A109-A490D58F15DD}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="16.85546875" customWidth="1"/>
@@ -795,59 +1199,78 @@
     <col min="3" max="3" width="12.140625" bestFit="1" customWidth="1"/>
     <col min="4" max="4" width="17.85546875" bestFit="1" customWidth="1"/>
     <col min="5" max="5" width="8.5703125" style="1" customWidth="1"/>
+    <col min="6" max="7" width="17.85546875" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-    </row>
-    <row r="2" spans="1:5" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" ht="4.5" customHeight="1" thickBot="1" x14ac:dyDescent="0.4">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
       <c r="E2" s="3"/>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="A3" s="13" t="s">
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" s="2" customFormat="1" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A3" s="18" t="s">
         <v>0</v>
       </c>
-      <c r="B3" s="14" t="s">
+      <c r="B3" s="19" t="s">
         <v>1</v>
       </c>
-      <c r="C3" s="14" t="s">
+      <c r="C3" s="19" t="s">
         <v>16</v>
       </c>
-      <c r="D3" s="21" t="s">
+      <c r="D3" s="20" t="s">
         <v>17</v>
       </c>
-      <c r="E3" s="15" t="s">
+      <c r="E3" s="21" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" s="10" t="s">
+      <c r="F3" s="20" t="s">
+        <v>24</v>
+      </c>
+      <c r="G3" s="20" t="s">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="A4" s="14" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="11" t="s">
+      <c r="B4" s="15" t="s">
         <v>2</v>
       </c>
-      <c r="C4" s="12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="22">
+      <c r="C4" s="16" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="17">
         <v>25.9</v>
       </c>
-      <c r="E4" s="17">
+      <c r="E4" s="15">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F4" s="17">
+        <f>D4*E4</f>
+        <v>310.79999999999995</v>
+      </c>
+      <c r="G4" s="22">
+        <f>F4*$D$25</f>
+        <v>15.54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A5" s="6" t="s">
         <v>15</v>
       </c>
@@ -857,14 +1280,22 @@
       <c r="C5" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D5" s="23">
+      <c r="D5" s="11">
         <v>29.9</v>
       </c>
-      <c r="E5" s="18">
+      <c r="E5" s="5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F5" s="11">
+        <f t="shared" ref="F5:G23" si="0">D5*E5</f>
+        <v>299</v>
+      </c>
+      <c r="G5" s="22">
+        <f t="shared" ref="G5:G25" si="1">F5*$D$25</f>
+        <v>14.950000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A6" s="6" t="s">
         <v>15</v>
       </c>
@@ -874,14 +1305,22 @@
       <c r="C6" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D6" s="23">
+      <c r="D6" s="11">
         <v>32.9</v>
       </c>
-      <c r="E6" s="18">
+      <c r="E6" s="5">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F6" s="11">
+        <f t="shared" si="0"/>
+        <v>197.39999999999998</v>
+      </c>
+      <c r="G6" s="22">
+        <f t="shared" si="1"/>
+        <v>9.8699999999999992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A7" s="6" t="s">
         <v>5</v>
       </c>
@@ -891,14 +1330,22 @@
       <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="23">
+      <c r="D7" s="11">
         <v>399.9</v>
       </c>
-      <c r="E7" s="18">
+      <c r="E7" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F7" s="11">
+        <f t="shared" si="0"/>
+        <v>1199.6999999999998</v>
+      </c>
+      <c r="G7" s="22">
+        <f t="shared" si="1"/>
+        <v>59.984999999999992</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A8" s="6" t="s">
         <v>6</v>
       </c>
@@ -908,14 +1355,22 @@
       <c r="C8" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D8" s="23">
+      <c r="D8" s="11">
         <v>249.9</v>
       </c>
-      <c r="E8" s="18">
+      <c r="E8" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F8" s="11">
+        <f t="shared" si="0"/>
+        <v>249.9</v>
+      </c>
+      <c r="G8" s="22">
+        <f t="shared" si="1"/>
+        <v>12.495000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A9" s="6" t="s">
         <v>6</v>
       </c>
@@ -925,14 +1380,22 @@
       <c r="C9" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D9" s="23">
+      <c r="D9" s="11">
         <v>259.89999999999998</v>
       </c>
-      <c r="E9" s="18">
+      <c r="E9" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F9" s="11">
+        <f t="shared" si="0"/>
+        <v>519.79999999999995</v>
+      </c>
+      <c r="G9" s="22">
+        <f t="shared" si="1"/>
+        <v>25.99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A10" s="6" t="s">
         <v>6</v>
       </c>
@@ -942,14 +1405,22 @@
       <c r="C10" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D10" s="23">
+      <c r="D10" s="11">
         <v>299.89999999999998</v>
       </c>
-      <c r="E10" s="18">
+      <c r="E10" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F10" s="11">
+        <f t="shared" si="0"/>
+        <v>299.89999999999998</v>
+      </c>
+      <c r="G10" s="22">
+        <f t="shared" si="1"/>
+        <v>14.994999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A11" s="6" t="s">
         <v>7</v>
       </c>
@@ -959,14 +1430,22 @@
       <c r="C11" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D11" s="23">
+      <c r="D11" s="11">
         <v>85.9</v>
       </c>
-      <c r="E11" s="18">
+      <c r="E11" s="5">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F11" s="11">
+        <f t="shared" si="0"/>
+        <v>687.2</v>
+      </c>
+      <c r="G11" s="22">
+        <f t="shared" si="1"/>
+        <v>34.360000000000007</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A12" s="6" t="s">
         <v>7</v>
       </c>
@@ -976,14 +1455,22 @@
       <c r="C12" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D12" s="23">
+      <c r="D12" s="11">
         <v>89.9</v>
       </c>
-      <c r="E12" s="18">
+      <c r="E12" s="5">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F12" s="11">
+        <f t="shared" si="0"/>
+        <v>449.5</v>
+      </c>
+      <c r="G12" s="22">
+        <f t="shared" si="1"/>
+        <v>22.475000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A13" s="6" t="s">
         <v>7</v>
       </c>
@@ -993,14 +1480,22 @@
       <c r="C13" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D13" s="23">
+      <c r="D13" s="11">
         <v>92.9</v>
       </c>
-      <c r="E13" s="18">
+      <c r="E13" s="5">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F13" s="11">
+        <f t="shared" si="0"/>
+        <v>557.40000000000009</v>
+      </c>
+      <c r="G13" s="22">
+        <f t="shared" si="1"/>
+        <v>27.870000000000005</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A14" s="6" t="s">
         <v>8</v>
       </c>
@@ -1010,14 +1505,22 @@
       <c r="C14" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D14" s="23">
+      <c r="D14" s="11">
         <v>149.9</v>
       </c>
-      <c r="E14" s="18">
+      <c r="E14" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F14" s="11">
+        <f t="shared" si="0"/>
+        <v>299.8</v>
+      </c>
+      <c r="G14" s="22">
+        <f t="shared" si="1"/>
+        <v>14.990000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A15" s="6" t="s">
         <v>9</v>
       </c>
@@ -1027,14 +1530,22 @@
       <c r="C15" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D15" s="23">
+      <c r="D15" s="11">
         <v>65.900000000000006</v>
       </c>
-      <c r="E15" s="18">
+      <c r="E15" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F15" s="11">
+        <f t="shared" si="0"/>
+        <v>790.80000000000007</v>
+      </c>
+      <c r="G15" s="22">
+        <f t="shared" si="1"/>
+        <v>39.540000000000006</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A16" s="6" t="s">
         <v>9</v>
       </c>
@@ -1044,14 +1555,22 @@
       <c r="C16" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D16" s="23">
+      <c r="D16" s="11">
         <v>69.900000000000006</v>
       </c>
-      <c r="E16" s="18">
+      <c r="E16" s="5">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F16" s="11">
+        <f t="shared" si="0"/>
+        <v>1048.5</v>
+      </c>
+      <c r="G16" s="22">
+        <f t="shared" si="1"/>
+        <v>52.425000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A17" s="6" t="s">
         <v>9</v>
       </c>
@@ -1061,14 +1580,22 @@
       <c r="C17" s="4" t="s">
         <v>18</v>
       </c>
-      <c r="D17" s="23">
+      <c r="D17" s="11">
         <v>70.900000000000006</v>
       </c>
-      <c r="E17" s="18">
+      <c r="E17" s="5">
         <v>13</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F17" s="11">
+        <f t="shared" si="0"/>
+        <v>921.7</v>
+      </c>
+      <c r="G17" s="22">
+        <f t="shared" si="1"/>
+        <v>46.085000000000008</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A18" s="6" t="s">
         <v>10</v>
       </c>
@@ -1078,14 +1605,22 @@
       <c r="C18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="23">
+      <c r="D18" s="11">
         <v>199.9</v>
       </c>
-      <c r="E18" s="18">
+      <c r="E18" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F18" s="11">
+        <f t="shared" si="0"/>
+        <v>399.8</v>
+      </c>
+      <c r="G18" s="22">
+        <f t="shared" si="1"/>
+        <v>19.990000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A19" s="6" t="s">
         <v>10</v>
       </c>
@@ -1095,14 +1630,22 @@
       <c r="C19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="23">
+      <c r="D19" s="11">
         <v>249.9</v>
       </c>
-      <c r="E19" s="18">
+      <c r="E19" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F19" s="11">
+        <f t="shared" si="0"/>
+        <v>249.9</v>
+      </c>
+      <c r="G19" s="22">
+        <f t="shared" si="1"/>
+        <v>12.495000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A20" s="6" t="s">
         <v>10</v>
       </c>
@@ -1112,14 +1655,22 @@
       <c r="C20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="23">
+      <c r="D20" s="11">
         <v>259.89999999999998</v>
       </c>
-      <c r="E20" s="18">
+      <c r="E20" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F20" s="11">
+        <f t="shared" si="0"/>
+        <v>0</v>
+      </c>
+      <c r="G20" s="22">
+        <f t="shared" si="1"/>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A21" s="6" t="s">
         <v>11</v>
       </c>
@@ -1129,14 +1680,22 @@
       <c r="C21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="23">
+      <c r="D21" s="11">
         <v>259.89999999999998</v>
       </c>
-      <c r="E21" s="18">
+      <c r="E21" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
+      <c r="F21" s="11">
+        <f t="shared" si="0"/>
+        <v>259.89999999999998</v>
+      </c>
+      <c r="G21" s="22">
+        <f t="shared" si="1"/>
+        <v>12.994999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A22" s="6" t="s">
         <v>12</v>
       </c>
@@ -1146,14 +1705,22 @@
       <c r="C22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="23">
-        <v>39.9</v>
-      </c>
-      <c r="E22" s="18">
+      <c r="D22" s="11">
+        <v>139.9</v>
+      </c>
+      <c r="E22" s="5">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
+      <c r="F22" s="11">
+        <f t="shared" si="0"/>
+        <v>1538.9</v>
+      </c>
+      <c r="G22" s="22">
+        <f t="shared" si="1"/>
+        <v>76.945000000000007</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" ht="15.75" thickBot="1" x14ac:dyDescent="0.3">
       <c r="A23" s="7" t="s">
         <v>13</v>
       </c>
@@ -1163,26 +1730,63 @@
       <c r="C23" s="9" t="s">
         <v>19</v>
       </c>
-      <c r="D23" s="24">
+      <c r="D23" s="12">
         <v>49.9</v>
       </c>
-      <c r="E23" s="19">
+      <c r="E23" s="8">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="D24" s="25">
+      <c r="F23" s="12">
+        <f t="shared" si="0"/>
+        <v>1047.8999999999999</v>
+      </c>
+      <c r="G23" s="22">
+        <f t="shared" si="1"/>
+        <v>52.394999999999996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A24" s="28" t="s">
+        <v>25</v>
+      </c>
+      <c r="B24" s="29"/>
+      <c r="C24" s="29"/>
+      <c r="D24" s="30">
         <f>SUM(D4:D23)</f>
-        <v>2983.0000000000009</v>
-      </c>
-      <c r="E24" s="1">
+        <v>3083.0000000000009</v>
+      </c>
+      <c r="E24" s="31">
         <f>SUM(E4:E23)</f>
         <v>132</v>
       </c>
+      <c r="F24" s="32">
+        <f>SUM(F4:F23)</f>
+        <v>11327.8</v>
+      </c>
+      <c r="G24" s="36">
+        <f t="shared" si="1"/>
+        <v>566.39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="19.5" thickBot="1" x14ac:dyDescent="0.35">
+      <c r="A25" s="26" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="27"/>
+      <c r="C25" s="27"/>
+      <c r="D25" s="33">
+        <v>0.05</v>
+      </c>
+      <c r="E25" s="34"/>
+      <c r="F25" s="34"/>
+      <c r="G25" s="35"/>
     </row>
   </sheetData>
-  <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+  <mergeCells count="4">
+    <mergeCell ref="A25:C25"/>
+    <mergeCell ref="D25:G25"/>
+    <mergeCell ref="A1:G1"/>
+    <mergeCell ref="A24:C24"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
 </worksheet>
@@ -1190,33 +1794,39 @@
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{D1525D4F-4FEE-4357-9658-5E1916B70D88}">
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="14.85546875" bestFit="1" customWidth="1"/>
-    <col min="2" max="2" width="15.28515625" style="1" bestFit="1" customWidth="1"/>
-    <col min="3" max="3" width="15.5703125" bestFit="1" customWidth="1"/>
-    <col min="4" max="4" width="21" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="9.42578125" style="1" bestFit="1" customWidth="1"/>
+    <col min="1" max="1" width="16.140625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="16.140625" style="1" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="16.7109375" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="22.42578125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="10.7109375" style="1" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="18.28515625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="23.7109375" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:5" ht="21" x14ac:dyDescent="0.35">
-      <c r="A1" s="26" t="s">
+    <row r="1" spans="1:7" ht="21" x14ac:dyDescent="0.35">
+      <c r="A1" s="13" t="s">
         <v>21</v>
       </c>
-      <c r="B1" s="26"/>
-      <c r="C1" s="26"/>
-      <c r="D1" s="26"/>
-      <c r="E1" s="26"/>
-    </row>
-    <row r="2" spans="1:5" ht="4.5" customHeight="1" x14ac:dyDescent="0.35">
+      <c r="B1" s="13"/>
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="E1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+    </row>
+    <row r="2" spans="1:7" ht="4.5" customHeight="1" x14ac:dyDescent="0.35">
       <c r="A2" s="3"/>
       <c r="B2" s="3"/>
       <c r="C2" s="3"/>
       <c r="D2" s="3"/>
-      <c r="E2" s="20"/>
-    </row>
-    <row r="3" spans="1:5" s="2" customFormat="1" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="E2" s="10"/>
+      <c r="F2" s="3"/>
+      <c r="G2" s="3"/>
+    </row>
+    <row r="3" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
       <c r="A3" s="2" t="s">
         <v>0</v>
       </c>
@@ -1232,363 +1842,552 @@
       <c r="E3" s="2" t="s">
         <v>22</v>
       </c>
-    </row>
-    <row r="4" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A4" t="s">
+      <c r="F3" s="2" t="s">
+        <v>28</v>
+      </c>
+      <c r="G3" s="2" t="s">
+        <v>29</v>
+      </c>
+    </row>
+    <row r="4" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A4" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B4" s="1" t="s">
+      <c r="B4" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C4" t="s">
-        <v>18</v>
-      </c>
-      <c r="D4" s="16">
+      <c r="C4" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D4" s="11">
         <v>25.9</v>
       </c>
-      <c r="E4" s="1">
+      <c r="E4" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="5" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A5" t="s">
+      <c r="F4" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>310.79999999999995</v>
+      </c>
+      <c r="G4" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>15.54</v>
+      </c>
+    </row>
+    <row r="5" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A5" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B5" s="1" t="s">
+      <c r="B5" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C5" t="s">
-        <v>18</v>
-      </c>
-      <c r="D5" s="16">
+      <c r="C5" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D5" s="11">
         <v>29.9</v>
       </c>
-      <c r="E5" s="1">
+      <c r="E5" s="5">
         <v>10</v>
       </c>
-    </row>
-    <row r="6" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A6" t="s">
+      <c r="F5" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>299</v>
+      </c>
+      <c r="G5" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>14.950000000000001</v>
+      </c>
+    </row>
+    <row r="6" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A6" s="4" t="s">
         <v>15</v>
       </c>
-      <c r="B6" s="1" t="s">
+      <c r="B6" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C6" t="s">
-        <v>18</v>
-      </c>
-      <c r="D6" s="16">
+      <c r="C6" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D6" s="11">
         <v>32.9</v>
       </c>
-      <c r="E6" s="1">
+      <c r="E6" s="5">
         <v>6</v>
       </c>
-    </row>
-    <row r="7" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A7" t="s">
+      <c r="F6" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>197.39999999999998</v>
+      </c>
+      <c r="G6" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>9.8699999999999992</v>
+      </c>
+    </row>
+    <row r="7" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A7" s="4" t="s">
         <v>5</v>
       </c>
-      <c r="B7" s="1" t="s">
+      <c r="B7" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C7" t="s">
+      <c r="C7" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D7" s="16">
+      <c r="D7" s="11">
         <v>399.9</v>
       </c>
-      <c r="E7" s="1">
+      <c r="E7" s="5">
         <v>3</v>
       </c>
-    </row>
-    <row r="8" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A8" t="s">
+      <c r="F7" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>1199.6999999999998</v>
+      </c>
+      <c r="G7" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>59.984999999999992</v>
+      </c>
+    </row>
+    <row r="8" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A8" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B8" s="1" t="s">
+      <c r="B8" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C8" t="s">
-        <v>18</v>
-      </c>
-      <c r="D8" s="16">
+      <c r="C8" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D8" s="11">
         <v>249.9</v>
       </c>
-      <c r="E8" s="1">
+      <c r="E8" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A9" t="s">
+      <c r="F8" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>249.9</v>
+      </c>
+      <c r="G8" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>12.495000000000001</v>
+      </c>
+    </row>
+    <row r="9" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A9" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B9" s="1" t="s">
+      <c r="B9" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C9" t="s">
-        <v>18</v>
-      </c>
-      <c r="D9" s="16">
+      <c r="C9" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D9" s="11">
         <v>259.89999999999998</v>
       </c>
-      <c r="E9" s="1">
+      <c r="E9" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="10" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A10" t="s">
+      <c r="F9" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>519.79999999999995</v>
+      </c>
+      <c r="G9" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>25.99</v>
+      </c>
+    </row>
+    <row r="10" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A10" s="4" t="s">
         <v>6</v>
       </c>
-      <c r="B10" s="1" t="s">
+      <c r="B10" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C10" t="s">
-        <v>18</v>
-      </c>
-      <c r="D10" s="16">
+      <c r="C10" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D10" s="11">
         <v>299.89999999999998</v>
       </c>
-      <c r="E10" s="1">
+      <c r="E10" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="11" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A11" t="s">
+      <c r="F10" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>299.89999999999998</v>
+      </c>
+      <c r="G10" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>14.994999999999999</v>
+      </c>
+    </row>
+    <row r="11" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A11" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B11" s="1" t="s">
+      <c r="B11" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C11" t="s">
-        <v>18</v>
-      </c>
-      <c r="D11" s="16">
+      <c r="C11" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D11" s="11">
         <v>85.9</v>
       </c>
-      <c r="E11" s="1">
+      <c r="E11" s="5">
         <v>8</v>
       </c>
-    </row>
-    <row r="12" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A12" t="s">
+      <c r="F11" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>687.2</v>
+      </c>
+      <c r="G11" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>34.360000000000007</v>
+      </c>
+    </row>
+    <row r="12" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A12" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B12" s="1" t="s">
+      <c r="B12" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C12" t="s">
-        <v>18</v>
-      </c>
-      <c r="D12" s="16">
+      <c r="C12" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D12" s="11">
         <v>89.9</v>
       </c>
-      <c r="E12" s="1">
+      <c r="E12" s="5">
         <v>5</v>
       </c>
-    </row>
-    <row r="13" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A13" t="s">
+      <c r="F12" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>449.5</v>
+      </c>
+      <c r="G12" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>22.475000000000001</v>
+      </c>
+    </row>
+    <row r="13" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A13" s="4" t="s">
         <v>7</v>
       </c>
-      <c r="B13" s="1" t="s">
+      <c r="B13" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C13" t="s">
-        <v>18</v>
-      </c>
-      <c r="D13" s="16">
+      <c r="C13" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D13" s="11">
         <v>92.9</v>
       </c>
-      <c r="E13" s="1">
+      <c r="E13" s="5">
         <v>6</v>
       </c>
-    </row>
-    <row r="14" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A14" t="s">
+      <c r="F13" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>557.40000000000009</v>
+      </c>
+      <c r="G13" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>27.870000000000005</v>
+      </c>
+    </row>
+    <row r="14" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A14" s="4" t="s">
         <v>8</v>
       </c>
-      <c r="B14" s="1" t="s">
+      <c r="B14" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C14" t="s">
-        <v>18</v>
-      </c>
-      <c r="D14" s="16">
+      <c r="C14" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D14" s="11">
         <v>149.9</v>
       </c>
-      <c r="E14" s="1">
+      <c r="E14" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="15" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A15" t="s">
+      <c r="F14" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>299.8</v>
+      </c>
+      <c r="G14" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>14.990000000000002</v>
+      </c>
+    </row>
+    <row r="15" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A15" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B15" s="1" t="s">
+      <c r="B15" s="5" t="s">
         <v>2</v>
       </c>
-      <c r="C15" t="s">
-        <v>18</v>
-      </c>
-      <c r="D15" s="16">
+      <c r="C15" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D15" s="11">
         <v>65.900000000000006</v>
       </c>
-      <c r="E15" s="1">
+      <c r="E15" s="5">
         <v>12</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A16" t="s">
+      <c r="F15" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>790.80000000000007</v>
+      </c>
+      <c r="G15" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>39.540000000000006</v>
+      </c>
+    </row>
+    <row r="16" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A16" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B16" s="1" t="s">
+      <c r="B16" s="5" t="s">
         <v>3</v>
       </c>
-      <c r="C16" t="s">
-        <v>18</v>
-      </c>
-      <c r="D16" s="16">
+      <c r="C16" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D16" s="11">
         <v>69.900000000000006</v>
       </c>
-      <c r="E16" s="1">
+      <c r="E16" s="5">
         <v>15</v>
       </c>
-    </row>
-    <row r="17" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A17" t="s">
+      <c r="F16" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>1048.5</v>
+      </c>
+      <c r="G16" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>52.425000000000004</v>
+      </c>
+    </row>
+    <row r="17" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A17" s="4" t="s">
         <v>9</v>
       </c>
-      <c r="B17" s="1" t="s">
+      <c r="B17" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="C17" t="s">
-        <v>18</v>
-      </c>
-      <c r="D17" s="16">
+      <c r="C17" s="4" t="s">
+        <v>18</v>
+      </c>
+      <c r="D17" s="11">
         <v>70.900000000000006</v>
       </c>
-      <c r="E17" s="1">
+      <c r="E17" s="5">
         <v>13</v>
       </c>
-    </row>
-    <row r="18" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A18" t="s">
+      <c r="F17" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>921.7</v>
+      </c>
+      <c r="G17" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>46.085000000000008</v>
+      </c>
+    </row>
+    <row r="18" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A18" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B18" s="1">
+      <c r="B18" s="5">
         <v>36</v>
       </c>
-      <c r="C18" t="s">
+      <c r="C18" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D18" s="16">
+      <c r="D18" s="11">
         <v>199.9</v>
       </c>
-      <c r="E18" s="1">
+      <c r="E18" s="5">
         <v>2</v>
       </c>
-    </row>
-    <row r="19" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A19" t="s">
+      <c r="F18" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>399.8</v>
+      </c>
+      <c r="G18" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>19.990000000000002</v>
+      </c>
+    </row>
+    <row r="19" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A19" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B19" s="1">
+      <c r="B19" s="5">
         <v>37</v>
       </c>
-      <c r="C19" t="s">
+      <c r="C19" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D19" s="16">
+      <c r="D19" s="11">
         <v>249.9</v>
       </c>
-      <c r="E19" s="1">
+      <c r="E19" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="20" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A20" t="s">
+      <c r="F19" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>249.9</v>
+      </c>
+      <c r="G19" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>12.495000000000001</v>
+      </c>
+    </row>
+    <row r="20" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A20" s="4" t="s">
         <v>10</v>
       </c>
-      <c r="B20" s="1">
+      <c r="B20" s="5">
         <v>38</v>
       </c>
-      <c r="C20" t="s">
+      <c r="C20" s="4" t="s">
         <v>20</v>
       </c>
-      <c r="D20" s="16">
+      <c r="D20" s="11">
         <v>259.89999999999998</v>
       </c>
-      <c r="E20" s="1">
+      <c r="E20" s="5">
         <v>0</v>
       </c>
-    </row>
-    <row r="21" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A21" t="s">
+      <c r="F20" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>0</v>
+      </c>
+      <c r="G20" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="21" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A21" s="4" t="s">
         <v>11</v>
       </c>
-      <c r="B21" s="1" t="s">
+      <c r="B21" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C21" t="s">
+      <c r="C21" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D21" s="16">
+      <c r="D21" s="11">
         <v>259.89999999999998</v>
       </c>
-      <c r="E21" s="1">
+      <c r="E21" s="5">
         <v>1</v>
       </c>
-    </row>
-    <row r="22" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A22" t="s">
+      <c r="F21" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>259.89999999999998</v>
+      </c>
+      <c r="G21" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>12.994999999999999</v>
+      </c>
+    </row>
+    <row r="22" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A22" s="4" t="s">
         <v>12</v>
       </c>
-      <c r="B22" s="1" t="s">
+      <c r="B22" s="5" t="s">
         <v>14</v>
       </c>
-      <c r="C22" t="s">
+      <c r="C22" s="4" t="s">
         <v>19</v>
       </c>
-      <c r="D22" s="16">
-        <v>39.9</v>
-      </c>
-      <c r="E22" s="1">
+      <c r="D22" s="11">
+        <v>139.9</v>
+      </c>
+      <c r="E22" s="5">
         <v>11</v>
       </c>
-    </row>
-    <row r="23" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A23" t="s">
+      <c r="F22" s="38">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>1538.9</v>
+      </c>
+      <c r="G22" s="38">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>76.945000000000007</v>
+      </c>
+    </row>
+    <row r="23" spans="1:7" x14ac:dyDescent="0.25">
+      <c r="A23" s="24" t="s">
         <v>13</v>
       </c>
-      <c r="B23" s="1" t="s">
+      <c r="B23" s="23" t="s">
         <v>14</v>
       </c>
-      <c r="C23" t="s">
+      <c r="C23" s="24" t="s">
         <v>19</v>
       </c>
-      <c r="D23" s="16">
+      <c r="D23" s="25">
         <v>49.9</v>
       </c>
-      <c r="E23" s="1">
+      <c r="E23" s="23">
         <v>21</v>
       </c>
-    </row>
-    <row r="24" spans="1:5" x14ac:dyDescent="0.25">
-      <c r="A24" t="s">
+      <c r="F23" s="42">
+        <f>Tabela5[[#This Row],[Preço Unitário]]*Tabela5[[#This Row],[Qtd]]</f>
+        <v>1047.8999999999999</v>
+      </c>
+      <c r="G23" s="42">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>52.394999999999996</v>
+      </c>
+    </row>
+    <row r="24" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A24" s="37" t="s">
         <v>23</v>
       </c>
-      <c r="D24" s="16">
-        <f>SUBTOTAL(109,Tabela5[Preço Unitário])</f>
-        <v>2983.0000000000009</v>
-      </c>
-      <c r="E24" s="1">
-        <f>SUBTOTAL(109,Tabela5[Qtd])</f>
+      <c r="B24" s="37"/>
+      <c r="C24" s="37"/>
+      <c r="D24" s="43">
+        <f>SUM(D4:D23)</f>
+        <v>3083.0000000000009</v>
+      </c>
+      <c r="E24" s="43">
+        <f>SUM(E4:E23)</f>
         <v>132</v>
       </c>
+      <c r="F24" s="43">
+        <f>SUM(F4:F23)</f>
+        <v>11327.8</v>
+      </c>
+      <c r="G24" s="43">
+        <f>Tabela5[[#This Row],[Valor Total]]*Tabela5[[#Totals],[Preço Unitário]]</f>
+        <v>566.39</v>
+      </c>
+    </row>
+    <row r="25" spans="1:7" ht="18.75" x14ac:dyDescent="0.3">
+      <c r="A25" s="37" t="s">
+        <v>26</v>
+      </c>
+      <c r="B25" s="37"/>
+      <c r="C25" s="37"/>
+      <c r="D25" s="39" t="s">
+        <v>30</v>
+      </c>
+      <c r="E25" s="40"/>
+      <c r="F25" s="41"/>
+      <c r="G25" s="40"/>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:E1"/>
+    <mergeCell ref="A1:G1"/>
   </mergeCells>
   <pageMargins left="0.511811024" right="0.511811024" top="0.78740157499999996" bottom="0.78740157499999996" header="0.31496062000000002" footer="0.31496062000000002"/>
   <tableParts count="1">

</xml_diff>